<commit_message>
Fixed bug in ProPricerExporter for old ProjectMap Fixed bug in Labor Type/Spread Importer for BRC Id being 0 Fixed Unit Tests
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Tests/ActionLogic/Import/MOQ Table/MOQTableSSC_Invalid.xlsx
+++ b/GenBOE/GenBOE.Tests/ActionLogic/Import/MOQ Table/MOQTableSSC_Invalid.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\Documents\Repos\IES\GenBOE\GenBOE.Tests\ActionLogic\Import\MOQ Table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\source\IES\GenBOE\GenBOE.Tests\ActionLogic\Import\MOQ Table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B2928B-7CB2-41B7-ABF4-2ED47789835D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A49C2A6F-8BA6-422C-A691-EE299647CD32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30585" yWindow="2205" windowWidth="21600" windowHeight="11385" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
+    <workbookView xWindow="2130" yWindow="0" windowWidth="19395" windowHeight="15480" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
   </bookViews>
   <sheets>
     <sheet name="MOQ Tables" sheetId="1" r:id="rId1"/>
@@ -126,9 +126,6 @@
     <t>Employee ID Filters</t>
   </si>
   <si>
-    <t>Total Relevant Hours After Employee ID Filters Applied</t>
-  </si>
-  <si>
     <t>Query Type</t>
   </si>
   <si>
@@ -277,6 +274,9 @@
   </si>
   <si>
     <t>FW 1/2021</t>
+  </si>
+  <si>
+    <t>Total Relevant Hours exclude unpaid (zero cost) hours and service centers, after application of Employee ID Filters</t>
   </si>
 </sst>
 </file>
@@ -462,9 +462,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -502,7 +502,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -608,7 +608,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -750,7 +750,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -804,767 +804,767 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J2" s="3">
         <v>100</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J3" s="3">
         <v>100</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J4" s="3">
         <v>100</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J5" s="3">
         <v>100</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="F6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J6" s="3">
         <v>100</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="I7" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J7" s="3">
         <v>100</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J8" s="3">
         <v>100</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J9" s="3">
         <v>100</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J10" s="3">
         <v>100</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="I11" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J11" s="3">
         <v>100</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="I12" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J12" s="3">
         <v>100</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="H13" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J13" s="3">
         <v>100</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G14" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="H14" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J14" s="3">
         <v>100</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="H15" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J15" s="3">
         <v>100</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="H16" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J16" s="3">
         <v>100</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G17" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="H17" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J17" s="3">
         <v>100</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J18" s="3">
         <v>100</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>53</v>
-      </c>
       <c r="C19" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="I19" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J19" s="3">
         <v>100</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="D20" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="I20" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J20" s="3">
         <v>100</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J21" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>57</v>
-      </c>
       <c r="K21" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -1646,17 +1646,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>